<commit_message>
Cập nhật theo PO 25/10: N022/N117 PASS (grandfather ẩn My Balance là đúng), N125 chạy lại cài mới
</commit_message>
<xml_diff>
--- a/results/TC_IIP055.1.16_Daily_Quota_Topup_ket_qua_v2.xlsx
+++ b/results/TC_IIP055.1.16_Daily_Quota_Topup_ket_qua_v2.xlsx
@@ -2089,9 +2089,9 @@
 2. Nút "Get More" vẫn hiển thị</t>
         </is>
       </c>
-      <c r="I27" s="38" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="I27" s="34" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J27" s="35" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="K27" s="35" t="inlineStr">
         <is>
-          <t>Autotest vòng 2 24/10 · lượt r2fin-test04_grandfatherState-112203 · CHẤM TAY: Grandfather (tier=unlimitedV1): Setting KHÔNG có hàng My Balance (SettingsView.swift:84 ẩn cố ý với user gen v1) → không có 413 'Unlimited' + Get More như Expected. Có thể là lệch spec có chủ đích của dev — hỏi PO.</t>
+          <t>Autotest vòng 2 24/10 · lượt r2fin-test04_grandfatherState-112203 · CHẤM TAY: PO/tester chốt 25/10 13:10: grandfather bị ẩn My Balance là ĐÚNG. App ẩn hàng My Balance với grandfather (SettingsView.swift:84) — đúng hành vi đã chốt; Expected TC ('413 Unlimited + Get More') cần cập nhật.</t>
         </is>
       </c>
       <c r="L27" s="36" t="inlineStr">
@@ -7509,9 +7509,9 @@
 3. Lần Q + 1 gen bình thường, không hiện 481</t>
         </is>
       </c>
-      <c r="I126" s="38" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="I126" s="34" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J126" s="35" t="inlineStr">
@@ -7521,7 +7521,7 @@
       </c>
       <c r="K126" s="35" t="inlineStr">
         <is>
-          <t>Autotest vòng 2 24/10 · lượt r2fin-test04_grandfatherState-112203, r2fin-test06_grandfatherGenBeyondQ-112506</t>
+          <t>Autotest vòng 2 24/10 · lượt r2fin-test04_grandfatherState-112203, r2fin-test06_grandfatherGenBeyondQ-112506 · CHẤM TAY: PO/tester chốt 25/10 13:10: grandfather bị ẩn My Balance là ĐÚNG. Header badge ẩn, không nút Upgrade (N117-a) + gen Q+1 lần không 481 (N117-b, 21/21) — đạt; phần '413 hiển thị Unlimited' của Expected không áp dụng vì My Balance ẩn (cần cập nhật TC).</t>
         </is>
       </c>
       <c r="L126" s="36" t="inlineStr">
@@ -7896,12 +7896,12 @@
       </c>
       <c r="J133" s="35" t="inlineStr">
         <is>
-          <t>KQ: RC ép='empty' · giá trị app đang dùng=2026-10-24T00:00:00Z · tier=creditV3 · isUnlimitedGen=false · 413=0 · gen: 481, -</t>
+          <t>KQ: RC ép='empty' · giá trị app đang dùng=2026-08-11T00:00:00Z · tier=creditV3 · isUnlimitedGen=false · 413=0 · gen: 481, -</t>
         </is>
       </c>
       <c r="K133" s="35" t="inlineStr">
         <is>
-          <t>Autotest vòng 2 24/10 · lượt r2fin-rc-empty-124336 · CHẤM TAY: RC quota_grandfather_until rỗng (ép trong code, đi qua luật syncAllKeys): app bỏ qua chuỗi rỗng → giữ giá trị đã lưu 2026-10-24 (cài mới thì dùng default code 2026-08-11) → tier=creditV3, VẪN áp quota (ví 0 → 481). Expected: không áp quota cho ai. Code chủ ý ngược spec: GeniusApiVersionRouter.swift:99–101 'Rỗng hoặc parse fail → không grandfather ai' — hỏi PO chốt bên nào.</t>
+          <t>Autotest vòng 2 24/10 · lượt r2fin-n125-fresh2-131850 · CHẤM TAY: Chạy lại 25/10 13:13–13:20 CÀI MỚI (gỡ app → build RC quota_grandfather_until='' → cài): app bỏ qua chuỗi rỗng, dùng default code 2026-08-11T00:00:00Z → tier=creditV3, quotaEnforced=true; ví 0/0 → gen Enhance bị chặn 481 ngay ở Analyze. Lượt trước (không gỡ app) giữ giá trị cũ 2026-10-24 → cùng kết quả. Expected 'Lần Q+1 không bị chặn' → không đạt. (User ghi chú: đây là case check — kết quả đo được ở trên.)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bỏ 16 case cần giả lập phía server (N/A theo yêu cầu 25/10)
</commit_message>
<xml_diff>
--- a/results/TC_IIP055.1.16_Daily_Quota_Topup_ket_qua_v2.xlsx
+++ b/results/TC_IIP055.1.16_Daily_Quota_Topup_ket_qua_v2.xlsx
@@ -2436,13 +2436,13 @@
       </c>
       <c r="I33" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J33" s="35" t="inlineStr"/>
       <c r="K33" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -2927,13 +2927,13 @@
       </c>
       <c r="I42" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J42" s="35" t="inlineStr"/>
       <c r="K42" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -3280,13 +3280,13 @@
       </c>
       <c r="I48" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J48" s="35" t="inlineStr"/>
       <c r="K48" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -3334,13 +3334,13 @@
       </c>
       <c r="I49" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J49" s="35" t="inlineStr"/>
       <c r="K49" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -3387,13 +3387,13 @@
       </c>
       <c r="I50" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J50" s="35" t="inlineStr"/>
       <c r="K50" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -3492,13 +3492,13 @@
       </c>
       <c r="I52" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J52" s="35" t="inlineStr"/>
       <c r="K52" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -3879,13 +3879,13 @@
       </c>
       <c r="I59" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J59" s="35" t="inlineStr"/>
       <c r="K59" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -3931,13 +3931,13 @@
       </c>
       <c r="I60" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J60" s="35" t="inlineStr"/>
       <c r="K60" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -5266,13 +5266,13 @@
       </c>
       <c r="I84" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J84" s="35" t="inlineStr"/>
       <c r="K84" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -5317,13 +5317,13 @@
       </c>
       <c r="I85" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J85" s="35" t="inlineStr"/>
       <c r="K85" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -6281,13 +6281,13 @@
       </c>
       <c r="I102" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J102" s="35" t="inlineStr"/>
       <c r="K102" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -7333,13 +7333,13 @@
       </c>
       <c r="I122" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J122" s="35" t="inlineStr"/>
       <c r="K122" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -9519,13 +9519,13 @@
       </c>
       <c r="I167" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J167" s="35" t="inlineStr"/>
       <c r="K167" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần proxy bắt request offering</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -9569,13 +9569,13 @@
       </c>
       <c r="I168" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J168" s="35" t="inlineStr"/>
       <c r="K168" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần proxy bắt request lúc launch</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -9616,13 +9616,13 @@
       </c>
       <c r="I169" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J169" s="35" t="inlineStr"/>
       <c r="K169" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>
@@ -10025,13 +10025,13 @@
       </c>
       <c r="I177" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J177" s="35" t="inlineStr"/>
       <c r="K177" s="35" t="inlineStr">
         <is>
-          <t>Chờ BE/Infra: cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, proxy) — theo luật không tự giả lỗi server</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bỏ 3 case cần PO đổi CMS (N/A theo yêu cầu 25/10)
</commit_message>
<xml_diff>
--- a/results/TC_IIP055.1.16_Daily_Quota_Topup_ket_qua_v2.xlsx
+++ b/results/TC_IIP055.1.16_Daily_Quota_Topup_ket_qua_v2.xlsx
@@ -8443,13 +8443,13 @@
       </c>
       <c r="I145" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J145" s="35" t="inlineStr"/>
       <c r="K145" s="35" t="inlineStr">
         <is>
-          <t>Phần app: key daily_quota_amount đã gỡ khỏi RemoteConfigKeys.swift:216–218 (đọc code); 413=15 cần PO đặt Q=15 trên CMS — Chờ PO</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10: case cần PO đổi số lượt/ngày (Q) trên CMS.</t>
         </is>
       </c>
     </row>
@@ -8496,13 +8496,13 @@
       </c>
       <c r="I146" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J146" s="35" t="inlineStr"/>
       <c r="K146" s="35" t="inlineStr">
         <is>
-          <t>Chờ PO: đổi số lượt/ngày (Q) trên CMS</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10: case cần PO đổi số lượt/ngày (Q) trên CMS.</t>
         </is>
       </c>
     </row>
@@ -8604,13 +8604,13 @@
       </c>
       <c r="I148" s="41" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J148" s="35" t="inlineStr"/>
       <c r="K148" s="35" t="inlineStr">
         <is>
-          <t>Chờ PO: đổi số lượt/ngày (Q) trên CMS</t>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10: case cần PO đổi số lượt/ngày (Q) trên CMS.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bỏ 19 case khỏi phạm vi test (140 TC trong phạm vi)
</commit_message>
<xml_diff>
--- a/results/TC_IIP055.1.16_Daily_Quota_Topup_ket_qua_v2.xlsx
+++ b/results/TC_IIP055.1.16_Daily_Quota_Topup_ket_qua_v2.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Coverage" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Spec Q&amp;A" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Ngoài phạm vi" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -72,7 +73,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -145,6 +146,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -225,7 +231,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -346,6 +352,9 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2398,7 +2407,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="234" customHeight="1" s="25">
+    <row r="33" hidden="1" ht="234" customHeight="1" s="25">
       <c r="A33" s="31" t="n">
         <v>28</v>
       </c>
@@ -2434,9 +2443,9 @@
           <t>1. Thẻ không hiển thị số sai (không hiện 0 giả)</t>
         </is>
       </c>
-      <c r="I33" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I33" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J33" s="35" t="inlineStr"/>
@@ -2886,7 +2895,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="259.5" customHeight="1" s="25">
+    <row r="42" hidden="1" ht="259.5" customHeight="1" s="25">
       <c r="A42" s="31" t="n">
         <v>36</v>
       </c>
@@ -2925,9 +2934,9 @@
 2. Request không chứa field số dư (quota/topup/balance)</t>
         </is>
       </c>
-      <c r="I42" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I42" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J42" s="35" t="inlineStr"/>
@@ -3026,7 +3035,7 @@
 2. Không có câu cảnh báo nào về việc lượt bị tính</t>
         </is>
       </c>
-      <c r="I44" s="42" t="inlineStr">
+      <c r="I44" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -3088,7 +3097,7 @@
 3. Không hiển thị toast 483</t>
         </is>
       </c>
-      <c r="I45" s="42" t="inlineStr">
+      <c r="I45" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -3149,7 +3158,7 @@
           <t>1. quota_balance = Q − 1 (chỉ trừ 1 lần)</t>
         </is>
       </c>
-      <c r="I46" s="42" t="inlineStr">
+      <c r="I46" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -3211,7 +3220,7 @@
 3. quota_balance = Q − 1</t>
         </is>
       </c>
-      <c r="I47" s="43" t="inlineStr">
+      <c r="I47" s="44" t="inlineStr">
         <is>
           <t>Cần xem</t>
         </is>
@@ -3232,7 +3241,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="312" customHeight="1" s="25">
+    <row r="48" hidden="1" ht="312" customHeight="1" s="25">
       <c r="A48" s="31" t="n">
         <v>42</v>
       </c>
@@ -3278,9 +3287,9 @@
 3. BE ghi log CANCELLED_VENDOR_FAIL</t>
         </is>
       </c>
-      <c r="I48" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I48" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J48" s="35" t="inlineStr"/>
@@ -3290,7 +3299,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="399.75" customHeight="1" s="25">
+    <row r="49" hidden="1" ht="399.75" customHeight="1" s="25">
       <c r="A49" s="31" t="n">
         <v>43</v>
       </c>
@@ -3332,9 +3341,9 @@
 2. topup_balance = 1, quota_balance = Q (hoàn đúng ví topup)</t>
         </is>
       </c>
-      <c r="I49" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I49" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J49" s="35" t="inlineStr"/>
@@ -3344,7 +3353,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="351" customHeight="1" s="25">
+    <row r="50" hidden="1" ht="351" customHeight="1" s="25">
       <c r="A50" s="31" t="n">
         <v>44</v>
       </c>
@@ -3385,9 +3394,9 @@
 2. quota_balance = Q, topup_balance = 0</t>
         </is>
       </c>
-      <c r="I50" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I50" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J50" s="35" t="inlineStr"/>
@@ -3449,7 +3458,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="351" customHeight="1" s="25">
+    <row r="52" hidden="1" ht="351" customHeight="1" s="25">
       <c r="A52" s="31" t="n">
         <v>46</v>
       </c>
@@ -3490,9 +3499,9 @@
 2. quota_balance = Q</t>
         </is>
       </c>
-      <c r="I52" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I52" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J52" s="35" t="inlineStr"/>
@@ -3840,7 +3849,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="220.5" customHeight="1" s="25">
+    <row r="59" hidden="1" ht="220.5" customHeight="1" s="25">
       <c r="A59" s="31" t="n">
         <v>53</v>
       </c>
@@ -3877,9 +3886,9 @@
 2. Không tạo HOLD, số dư không đổi</t>
         </is>
       </c>
-      <c r="I59" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I59" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J59" s="35" t="inlineStr"/>
@@ -3889,7 +3898,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="324.75" customHeight="1" s="25">
+    <row r="60" hidden="1" ht="324.75" customHeight="1" s="25">
       <c r="A60" s="31" t="n">
         <v>54</v>
       </c>
@@ -3929,9 +3938,9 @@
 3. quota_balance không xuống âm</t>
         </is>
       </c>
-      <c r="I60" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I60" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J60" s="35" t="inlineStr"/>
@@ -4170,7 +4179,7 @@
 4. Không có đồng hồ đếm ngược, không có câu nói bao giờ lượt về</t>
         </is>
       </c>
-      <c r="I65" s="42" t="inlineStr">
+      <c r="I65" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -4619,7 +4628,7 @@
 5. Không có chữ "credit", "Unlimited", không có dòng nhắc thứ tự tiêu</t>
         </is>
       </c>
-      <c r="I73" s="42" t="inlineStr">
+      <c r="I73" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -4685,7 +4694,7 @@
 3. một công thức duy nhất' ghi màn topup = topup+quota</t>
         </is>
       </c>
-      <c r="I74" s="42" t="inlineStr">
+      <c r="I74" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -5226,7 +5235,7 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="273" customHeight="1" s="25">
+    <row r="84" hidden="1" ht="273" customHeight="1" s="25">
       <c r="A84" s="31" t="n">
         <v>76</v>
       </c>
@@ -5264,9 +5273,9 @@
           <t>1. 413 hiển thị topup +1 ngay (không chờ webhook)</t>
         </is>
       </c>
-      <c r="I84" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I84" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J84" s="35" t="inlineStr"/>
@@ -5276,7 +5285,7 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="259.5" customHeight="1" s="25">
+    <row r="85" hidden="1" ht="259.5" customHeight="1" s="25">
       <c r="A85" s="31" t="n">
         <v>77</v>
       </c>
@@ -5315,9 +5324,9 @@
           <t>1. topup_balance = 1 (không phải 2 hay 3)</t>
         </is>
       </c>
-      <c r="I85" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I85" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J85" s="35" t="inlineStr"/>
@@ -5369,7 +5378,7 @@
 2. Flow gen dở không được khôi phục, user phải chọn lại ảnh</t>
         </is>
       </c>
-      <c r="I86" s="42" t="inlineStr">
+      <c r="I86" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -5497,18 +5506,18 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="181.5" customFormat="1" customHeight="1" s="44">
-      <c r="A89" s="45" t="n">
+    <row r="89" ht="181.5" customFormat="1" customHeight="1" s="45">
+      <c r="A89" s="46" t="n">
         <v>82</v>
       </c>
       <c r="B89" s="37" t="n"/>
       <c r="C89" s="37" t="n"/>
-      <c r="D89" s="46" t="inlineStr">
+      <c r="D89" s="47" t="inlineStr">
         <is>
           <t>Grandfather mua topup — mua bình thường, lượt nằm nguyên trong ví</t>
         </is>
       </c>
-      <c r="E89" s="47" t="inlineStr">
+      <c r="E89" s="48" t="inlineStr">
         <is>
           <t>1. RC (Firebase): enable_daily_quota = true · enable_topup = true · topup_offer_max_per_day = 1
 2. CMS: số lượt/ngày = Q (PO cấu hình trên CMS, mặc định 20; mọi số lượt trong TC tính theo Q)
@@ -5516,17 +5525,17 @@
 4. Có kết nối internet ổn định</t>
         </is>
       </c>
-      <c r="F89" s="47" t="inlineStr">
+      <c r="F89" s="48" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="G89" s="47" t="inlineStr">
+      <c r="G89" s="48" t="inlineStr">
         <is>
           <t>1. Gen thành công 3 lần</t>
         </is>
       </c>
-      <c r="H89" s="47" t="inlineStr">
+      <c r="H89" s="48" t="inlineStr">
         <is>
           <t>1. Không hiện số lượt quota trên badge
 2. Gen unlimited</t>
@@ -5658,7 +5667,7 @@
 </t>
         </is>
       </c>
-      <c r="I92" s="42" t="inlineStr">
+      <c r="I92" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -5848,7 +5857,7 @@
           <t>1. có hiện Last-chance rồi mới đến màn topup 216</t>
         </is>
       </c>
-      <c r="I95" s="43" t="inlineStr">
+      <c r="I95" s="44" t="inlineStr">
         <is>
           <t>Cần xem</t>
         </is>
@@ -6239,7 +6248,7 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="298.5" customHeight="1" s="25">
+    <row r="102" hidden="1" ht="298.5" customHeight="1" s="25">
       <c r="A102" s="31" t="n">
         <v>94</v>
       </c>
@@ -6279,9 +6288,9 @@
 2. Lần retry: vẫn hiện paywall feature và Last-chance trước khi gen</t>
         </is>
       </c>
-      <c r="I102" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I102" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J102" s="35" t="inlineStr"/>
@@ -7289,7 +7298,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="399.75" customHeight="1" s="25">
+    <row r="122" hidden="1" ht="399.75" customHeight="1" s="25">
       <c r="A122" s="31" t="n">
         <v>114</v>
       </c>
@@ -7331,9 +7340,9 @@
 2. Toast 483 hiển thị</t>
         </is>
       </c>
-      <c r="I122" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I122" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J122" s="35" t="inlineStr"/>
@@ -7906,7 +7915,7 @@
       </c>
     </row>
     <row r="134" ht="15.75" customHeight="1" s="25">
-      <c r="A134" s="48" t="inlineStr">
+      <c r="A134" s="49" t="inlineStr">
         <is>
           <t>▌ 11. Định danh App User ID</t>
         </is>
@@ -7955,7 +7964,7 @@
 2. Customer trên RevenueCat có đúng ID đó</t>
         </is>
       </c>
-      <c r="I135" s="43" t="inlineStr">
+      <c r="I135" s="44" t="inlineStr">
         <is>
           <t>Cần xem</t>
         </is>
@@ -8398,7 +8407,7 @@
         </is>
       </c>
     </row>
-    <row r="145" ht="246.75" customHeight="1" s="25">
+    <row r="145" hidden="1" ht="246.75" customHeight="1" s="25">
       <c r="A145" s="31" t="n">
         <v>136</v>
       </c>
@@ -8441,9 +8450,9 @@
 2. 413 hiển thị "15" (số lấy từ BE / CMS)</t>
         </is>
       </c>
-      <c r="I145" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I145" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J145" s="35" t="inlineStr"/>
@@ -8453,7 +8462,7 @@
         </is>
       </c>
     </row>
-    <row r="146" ht="207.75" customHeight="1" s="25">
+    <row r="146" hidden="1" ht="207.75" customHeight="1" s="25">
       <c r="A146" s="31" t="n">
         <v>137</v>
       </c>
@@ -8494,9 +8503,9 @@
 2. Lần gen vượt số lượt hiện 481</t>
         </is>
       </c>
-      <c r="I146" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I146" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J146" s="35" t="inlineStr"/>
@@ -8547,7 +8556,7 @@
 2. BE trả ERR12 cho request gọi thẳng</t>
         </is>
       </c>
-      <c r="I147" s="43" t="inlineStr">
+      <c r="I147" s="44" t="inlineStr">
         <is>
           <t>Cần xem</t>
         </is>
@@ -8563,7 +8572,7 @@
         </is>
       </c>
     </row>
-    <row r="148" ht="156" customHeight="1" s="25">
+    <row r="148" hidden="1" ht="156" customHeight="1" s="25">
       <c r="A148" s="31" t="n">
         <v>139</v>
       </c>
@@ -8602,9 +8611,9 @@
           <t>1. Mọi chỗ hiển thị đúng số lượt = giá trị Test data: "{giá trị} lần tạo mỗi ngày, làm mới tự động", "Chào mừng! Bạn có {giá trị} lần tạo mỗi ngày.", 482 "...cho bạn {giá trị} lần tạo mỗi ngày…"</t>
         </is>
       </c>
-      <c r="I148" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I148" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J148" s="35" t="inlineStr"/>
@@ -8777,7 +8786,7 @@
           <t>1. Không có badge, gen không bị chặn, không hiện 481</t>
         </is>
       </c>
-      <c r="I152" s="42" t="inlineStr">
+      <c r="I152" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -8833,7 +8842,7 @@
           <t xml:space="preserve">1. app không bị crash. </t>
         </is>
       </c>
-      <c r="I153" s="42" t="inlineStr">
+      <c r="I153" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -8883,7 +8892,7 @@
           <t>1. Get More 'luôn hiện', CTA 'Mua thêm' ở 481, màn topup offer xử lý thế nào khi tắt topup]</t>
         </is>
       </c>
-      <c r="I154" s="42" t="inlineStr">
+      <c r="I154" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -8997,7 +9006,7 @@
 </t>
         </is>
       </c>
-      <c r="I156" s="42" t="inlineStr">
+      <c r="I156" s="43" t="inlineStr">
         <is>
           <t>Lệch spec</t>
         </is>
@@ -9473,7 +9482,7 @@
         </is>
       </c>
     </row>
-    <row r="167" ht="220.5" customHeight="1" s="25">
+    <row r="167" hidden="1" ht="220.5" customHeight="1" s="25">
       <c r="A167" s="31" t="n">
         <v>158</v>
       </c>
@@ -9517,9 +9526,9 @@
           <t>1. Request tải offering 216_0.99 chỉ phát sinh khi mở màn topup</t>
         </is>
       </c>
-      <c r="I167" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I167" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J167" s="35" t="inlineStr"/>
@@ -9529,7 +9538,7 @@
         </is>
       </c>
     </row>
-    <row r="168" ht="64.5" customHeight="1" s="25">
+    <row r="168" hidden="1" ht="64.5" customHeight="1" s="25">
       <c r="A168" s="31" t="n">
         <v>159</v>
       </c>
@@ -9567,9 +9576,9 @@
 2. Không xuất hiện dialog hệ thống "Sign in to Apple Account"</t>
         </is>
       </c>
-      <c r="I168" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I168" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J168" s="35" t="inlineStr"/>
@@ -9579,7 +9588,7 @@
         </is>
       </c>
     </row>
-    <row r="169" ht="195" customHeight="1" s="25">
+    <row r="169" hidden="1" ht="195" customHeight="1" s="25">
       <c r="A169" s="31" t="n">
         <v>160</v>
       </c>
@@ -9614,9 +9623,9 @@
           <t>1. BE từ chối request, không tạo HOLD</t>
         </is>
       </c>
-      <c r="I169" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I169" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J169" s="35" t="inlineStr"/>
@@ -9985,7 +9994,7 @@
         </is>
       </c>
     </row>
-    <row r="177" ht="298.5" customHeight="1" s="25">
+    <row r="177" hidden="1" ht="298.5" customHeight="1" s="25">
       <c r="A177" s="31" t="n">
         <v>173</v>
       </c>
@@ -10023,9 +10032,9 @@
 2. App map ERR12 → hiện 481</t>
         </is>
       </c>
-      <c r="I177" s="41" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="I177" s="42" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
         </is>
       </c>
       <c r="J177" s="35" t="inlineStr"/>
@@ -10226,7 +10235,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="25">
-      <c r="A1" s="49" t="inlineStr">
+      <c r="A1" s="50" t="inlineStr">
         <is>
           <t>Quy ước Q, quota_grandfather_until và cách đưa ví về trạng thái cần test (không có công cụ seed)</t>
         </is>
@@ -10343,7 +10352,7 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
-      <c r="A12" s="49" t="inlineStr">
+      <c r="A12" s="50" t="inlineStr">
         <is>
           <t>Gom TC theo trạng thái ví ban đầu (setup 1 lần, chạy nhiều TC)</t>
         </is>
@@ -10554,7 +10563,7 @@
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="25">
-      <c r="A31" s="49" t="inlineStr">
+      <c r="A31" s="50" t="inlineStr">
         <is>
           <t>TC cần BE / Infra hỗ trợ (giả lập vendor, webhook, kiểm sổ BE, gọi API trực tiếp) — chưa chạy được bằng thao tác thật</t>
         </is>
@@ -10898,182 +10907,182 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="25">
-      <c r="A2" s="50" t="inlineStr">
+      <c r="A2" s="51" t="inlineStr">
         <is>
           <t>1. Home Header — Badge số lượt &amp; nút Upgrade / Get Pro</t>
         </is>
       </c>
-      <c r="B2" s="51" t="n">
+      <c r="B2" s="52" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="25">
-      <c r="A3" s="50" t="inlineStr">
+      <c r="A3" s="51" t="inlineStr">
         <is>
           <t>2. 410 Setting — dòng My Balance</t>
         </is>
       </c>
-      <c r="B3" s="51" t="n">
+      <c r="B3" s="52" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="25">
-      <c r="A4" s="50" t="inlineStr">
+      <c r="A4" s="51" t="inlineStr">
         <is>
           <t>3. 413 My Balance</t>
         </is>
       </c>
-      <c r="B4" s="51" t="n">
+      <c r="B4" s="52" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="25">
-      <c r="A5" s="50" t="inlineStr">
+      <c r="A5" s="51" t="inlineStr">
         <is>
           <t>4. Trừ lượt khi Gen (AC1)</t>
         </is>
       </c>
-      <c r="B5" s="51" t="n">
+      <c r="B5" s="52" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="25">
-      <c r="A6" s="50" t="inlineStr">
+      <c r="A6" s="51" t="inlineStr">
         <is>
           <t>5. 481 Dialog hết lượt</t>
         </is>
       </c>
-      <c r="B6" s="51" t="n">
+      <c r="B6" s="52" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="25">
-      <c r="A7" s="50" t="inlineStr">
+      <c r="A7" s="51" t="inlineStr">
         <is>
           <t>6. Màn topup &amp; mua Topup (AC2)</t>
         </is>
       </c>
-      <c r="B7" s="51" t="n">
+      <c r="B7" s="52" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="25">
-      <c r="A8" s="50" t="inlineStr">
+      <c r="A8" s="51" t="inlineStr">
         <is>
           <t>7. Luồng Free user (AC3)</t>
         </is>
       </c>
-      <c r="B8" s="51" t="n">
+      <c r="B8" s="52" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="25">
-      <c r="A9" s="50" t="inlineStr">
+      <c r="A9" s="51" t="inlineStr">
         <is>
           <t>8. 482 Mua thành công &amp; 483 Toast hoàn lượt</t>
         </is>
       </c>
-      <c r="B9" s="51" t="n">
+      <c r="B9" s="52" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="25">
-      <c r="A10" s="50" t="inlineStr">
+      <c r="A10" s="51" t="inlineStr">
         <is>
           <t>9. Reset quota hằng ngày</t>
         </is>
       </c>
-      <c r="B10" s="51" t="n">
+      <c r="B10" s="52" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
-      <c r="A11" s="50" t="inlineStr">
+      <c r="A11" s="51" t="inlineStr">
         <is>
           <t>10. Grandfather (AC4) — quota_grandfather_until</t>
         </is>
       </c>
-      <c r="B11" s="51" t="n">
+      <c r="B11" s="52" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
-      <c r="A12" s="50" t="inlineStr">
+      <c r="A12" s="51" t="inlineStr">
         <is>
           <t>11. Định danh App User ID</t>
         </is>
       </c>
-      <c r="B12" s="51" t="n">
+      <c r="B12" s="52" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
-      <c r="A13" s="50" t="inlineStr">
+      <c r="A13" s="51" t="inlineStr">
         <is>
           <t>12. Cấu hình số lượt/ngày trên CMS</t>
         </is>
       </c>
-      <c r="B13" s="51" t="n">
+      <c r="B13" s="52" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
-      <c r="A14" s="50" t="inlineStr">
+      <c r="A14" s="51" t="inlineStr">
         <is>
           <t>13. Remote Config (Firebase)</t>
         </is>
       </c>
-      <c r="B14" s="51" t="n">
+      <c r="B14" s="52" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
-      <c r="A15" s="50" t="inlineStr">
+      <c r="A15" s="51" t="inlineStr">
         <is>
           <t>14. Copy, Paywall &amp; Policy</t>
         </is>
       </c>
-      <c r="B15" s="51" t="n">
+      <c r="B15" s="52" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
-      <c r="A16" s="50" t="inlineStr">
+      <c r="A16" s="51" t="inlineStr">
         <is>
           <t>15. Non-functional</t>
         </is>
       </c>
-      <c r="B16" s="51" t="n">
+      <c r="B16" s="52" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
-      <c r="A17" s="50" t="inlineStr">
+      <c r="A17" s="51" t="inlineStr">
         <is>
           <t>16. Event tracking</t>
         </is>
       </c>
-      <c r="B17" s="51" t="n">
+      <c r="B17" s="52" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
-      <c r="A18" s="50" t="inlineStr">
+      <c r="A18" s="51" t="inlineStr">
         <is>
           <t>17. Regression / E2E</t>
         </is>
       </c>
-      <c r="B18" s="51" t="n">
+      <c r="B18" s="52" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
-      <c r="A19" s="52" t="inlineStr">
+      <c r="A19" s="53" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B19" s="53">
+      <c r="B19" s="54">
         <f>SUM(B2:B18)</f>
         <v/>
       </c>
@@ -11151,602 +11160,602 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="25">
-      <c r="A2" s="50" t="inlineStr">
+      <c r="A2" s="51" t="inlineStr">
         <is>
           <t>1. Home Header — Badge số lượt &amp; nút Upgrade / Get Pro</t>
         </is>
       </c>
-      <c r="B2" s="50" t="n">
+      <c r="B2" s="51" t="n">
         <v>14</v>
       </c>
-      <c r="C2" s="50" t="n">
+      <c r="C2" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="50" t="n">
+      <c r="D2" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="50" t="n">
+      <c r="E2" s="51" t="n">
         <v>10</v>
       </c>
-      <c r="F2" s="50" t="n">
+      <c r="F2" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="50" t="n">
+      <c r="G2" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="H2" s="50" t="n">
+      <c r="H2" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="54">
+      <c r="I2" s="55">
         <f>7/B2</f>
         <v/>
       </c>
-      <c r="J2" s="50" t="n">
+      <c r="J2" s="51" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="25">
-      <c r="A3" s="50" t="inlineStr">
+      <c r="A3" s="51" t="inlineStr">
         <is>
           <t>2. 410 Setting — dòng My Balance</t>
         </is>
       </c>
-      <c r="B3" s="50" t="n">
+      <c r="B3" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="50" t="n">
+      <c r="C3" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="50" t="n">
+      <c r="D3" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="50" t="n">
+      <c r="E3" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="50" t="n">
+      <c r="F3" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="50" t="n">
+      <c r="G3" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="50" t="n">
+      <c r="H3" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="54">
+      <c r="I3" s="55">
         <f>0/B3</f>
         <v/>
       </c>
-      <c r="J3" s="50" t="n">
+      <c r="J3" s="51" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="25">
-      <c r="A4" s="50" t="inlineStr">
+      <c r="A4" s="51" t="inlineStr">
         <is>
           <t>3. 413 My Balance</t>
         </is>
       </c>
-      <c r="B4" s="50" t="n">
+      <c r="B4" s="51" t="n">
         <v>11</v>
       </c>
-      <c r="C4" s="50" t="n">
+      <c r="C4" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="50" t="n">
+      <c r="D4" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="50" t="n">
+      <c r="E4" s="51" t="n">
         <v>7</v>
       </c>
-      <c r="F4" s="50" t="n">
+      <c r="F4" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="50" t="n">
+      <c r="G4" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="50" t="n">
+      <c r="H4" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="54">
+      <c r="I4" s="55">
         <f>3/B4</f>
         <v/>
       </c>
-      <c r="J4" s="50" t="n">
+      <c r="J4" s="51" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="25">
-      <c r="A5" s="50" t="inlineStr">
+      <c r="A5" s="51" t="inlineStr">
         <is>
           <t>4. Trừ lượt khi Gen (AC1)</t>
         </is>
       </c>
-      <c r="B5" s="50" t="n">
+      <c r="B5" s="51" t="n">
         <v>29</v>
       </c>
-      <c r="C5" s="50" t="n">
+      <c r="C5" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="50" t="n">
+      <c r="D5" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="50" t="n">
+      <c r="E5" s="51" t="n">
         <v>12</v>
       </c>
-      <c r="F5" s="50" t="n">
+      <c r="F5" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="50" t="n">
+      <c r="G5" s="51" t="n">
         <v>16</v>
       </c>
-      <c r="H5" s="50" t="n">
+      <c r="H5" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="54">
+      <c r="I5" s="55">
         <f>16/B5</f>
         <v/>
       </c>
-      <c r="J5" s="50" t="n">
+      <c r="J5" s="51" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="25">
-      <c r="A6" s="50" t="inlineStr">
+      <c r="A6" s="51" t="inlineStr">
         <is>
           <t>5. 481 Dialog hết lượt</t>
         </is>
       </c>
-      <c r="B6" s="50" t="n">
+      <c r="B6" s="51" t="n">
         <v>7</v>
       </c>
-      <c r="C6" s="50" t="n">
+      <c r="C6" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="50" t="n">
+      <c r="D6" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="50" t="n">
+      <c r="E6" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="F6" s="50" t="n">
+      <c r="F6" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="50" t="n">
+      <c r="G6" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="50" t="n">
+      <c r="H6" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="54">
+      <c r="I6" s="55">
         <f>2/B6</f>
         <v/>
       </c>
-      <c r="J6" s="50" t="n">
+      <c r="J6" s="51" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="25">
-      <c r="A7" s="50" t="inlineStr">
+      <c r="A7" s="51" t="inlineStr">
         <is>
           <t>6. Màn topup &amp; mua Topup (AC2)</t>
         </is>
       </c>
-      <c r="B7" s="50" t="n">
+      <c r="B7" s="51" t="n">
         <v>19</v>
       </c>
-      <c r="C7" s="50" t="n">
+      <c r="C7" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="50" t="n">
+      <c r="D7" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="50" t="n">
+      <c r="E7" s="51" t="n">
         <v>6</v>
       </c>
-      <c r="F7" s="50" t="n">
+      <c r="F7" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="50" t="n">
+      <c r="G7" s="51" t="n">
         <v>12</v>
       </c>
-      <c r="H7" s="50" t="n">
+      <c r="H7" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="54">
+      <c r="I7" s="55">
         <f>12/B7</f>
         <v/>
       </c>
-      <c r="J7" s="50" t="n">
+      <c r="J7" s="51" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="25">
-      <c r="A8" s="50" t="inlineStr">
+      <c r="A8" s="51" t="inlineStr">
         <is>
           <t>7. Luồng Free user (AC3)</t>
         </is>
       </c>
-      <c r="B8" s="50" t="n">
+      <c r="B8" s="51" t="n">
         <v>15</v>
       </c>
-      <c r="C8" s="50" t="n">
+      <c r="C8" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="50" t="n">
+      <c r="D8" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="50" t="n">
+      <c r="E8" s="51" t="n">
         <v>6</v>
       </c>
-      <c r="F8" s="50" t="n">
+      <c r="F8" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="50" t="n">
+      <c r="G8" s="51" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="50" t="n">
+      <c r="H8" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="54">
+      <c r="I8" s="55">
         <f>8/B8</f>
         <v/>
       </c>
-      <c r="J8" s="50" t="n">
+      <c r="J8" s="51" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="25">
-      <c r="A9" s="50" t="inlineStr">
+      <c r="A9" s="51" t="inlineStr">
         <is>
           <t>8. 482 Mua thành công &amp; 483 Toast hoàn lượt</t>
         </is>
       </c>
-      <c r="B9" s="50" t="n">
+      <c r="B9" s="51" t="n">
         <v>9</v>
       </c>
-      <c r="C9" s="50" t="n">
+      <c r="C9" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="50" t="n">
+      <c r="D9" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="50" t="n">
+      <c r="E9" s="51" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="50" t="n">
+      <c r="F9" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="50" t="n">
+      <c r="G9" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="H9" s="50" t="n">
+      <c r="H9" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I9" s="54">
+      <c r="I9" s="55">
         <f>3/B9</f>
         <v/>
       </c>
-      <c r="J9" s="50" t="n">
+      <c r="J9" s="51" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="25">
-      <c r="A10" s="50" t="inlineStr">
+      <c r="A10" s="51" t="inlineStr">
         <is>
           <t>9. Reset quota hằng ngày</t>
         </is>
       </c>
-      <c r="B10" s="50" t="n">
+      <c r="B10" s="51" t="n">
         <v>8</v>
       </c>
-      <c r="C10" s="50" t="n">
+      <c r="C10" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="50" t="n">
+      <c r="D10" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="50" t="n">
+      <c r="E10" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="50" t="n">
+      <c r="F10" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="50" t="n">
+      <c r="G10" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="50" t="n">
+      <c r="H10" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="54">
+      <c r="I10" s="55">
         <f>3/B10</f>
         <v/>
       </c>
-      <c r="J10" s="50" t="n">
+      <c r="J10" s="51" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
-      <c r="A11" s="50" t="inlineStr">
+      <c r="A11" s="51" t="inlineStr">
         <is>
           <t>10. Grandfather (AC4) — quota_grandfather_until</t>
         </is>
       </c>
-      <c r="B11" s="50" t="n">
+      <c r="B11" s="51" t="n">
         <v>10</v>
       </c>
-      <c r="C11" s="50" t="n">
+      <c r="C11" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="50" t="n">
+      <c r="D11" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="50" t="n">
+      <c r="E11" s="51" t="n">
         <v>9</v>
       </c>
-      <c r="F11" s="50" t="n">
+      <c r="F11" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="50" t="n">
+      <c r="G11" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="50" t="n">
+      <c r="H11" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="54">
+      <c r="I11" s="55">
         <f>1/B11</f>
         <v/>
       </c>
-      <c r="J11" s="50" t="n">
+      <c r="J11" s="51" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
-      <c r="A12" s="50" t="inlineStr">
+      <c r="A12" s="51" t="inlineStr">
         <is>
           <t>11. Định danh App User ID</t>
         </is>
       </c>
-      <c r="B12" s="50" t="n">
+      <c r="B12" s="51" t="n">
         <v>9</v>
       </c>
-      <c r="C12" s="50" t="n">
+      <c r="C12" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="50" t="n">
+      <c r="D12" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="50" t="n">
+      <c r="E12" s="51" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="50" t="n">
+      <c r="F12" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="50" t="n">
+      <c r="G12" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="50" t="n">
+      <c r="H12" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="54">
+      <c r="I12" s="55">
         <f>5/B12</f>
         <v/>
       </c>
-      <c r="J12" s="50" t="n">
+      <c r="J12" s="51" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
-      <c r="A13" s="50" t="inlineStr">
+      <c r="A13" s="51" t="inlineStr">
         <is>
           <t>12. Cấu hình số lượt/ngày trên CMS</t>
         </is>
       </c>
-      <c r="B13" s="50" t="n">
+      <c r="B13" s="51" t="n">
         <v>8</v>
       </c>
-      <c r="C13" s="50" t="n">
+      <c r="C13" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="50" t="n">
+      <c r="D13" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="50" t="n">
+      <c r="E13" s="51" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="50" t="n">
+      <c r="F13" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="50" t="n">
+      <c r="G13" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="50" t="n">
+      <c r="H13" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="54">
+      <c r="I13" s="55">
         <f>4/B13</f>
         <v/>
       </c>
-      <c r="J13" s="50" t="n">
+      <c r="J13" s="51" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
-      <c r="A14" s="50" t="inlineStr">
+      <c r="A14" s="51" t="inlineStr">
         <is>
           <t>13. Remote Config (Firebase)</t>
         </is>
       </c>
-      <c r="B14" s="50" t="n">
+      <c r="B14" s="51" t="n">
         <v>7</v>
       </c>
-      <c r="C14" s="50" t="n">
+      <c r="C14" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="50" t="n">
+      <c r="D14" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="50" t="n">
+      <c r="E14" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="50" t="n">
+      <c r="F14" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="G14" s="50" t="n">
+      <c r="G14" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="50" t="n">
+      <c r="H14" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="54">
+      <c r="I14" s="55">
         <f>5/B14</f>
         <v/>
       </c>
-      <c r="J14" s="50" t="n">
+      <c r="J14" s="51" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
-      <c r="A15" s="50" t="inlineStr">
+      <c r="A15" s="51" t="inlineStr">
         <is>
           <t>14. Copy, Paywall &amp; Policy</t>
         </is>
       </c>
-      <c r="B15" s="50" t="n">
+      <c r="B15" s="51" t="n">
         <v>8</v>
       </c>
-      <c r="C15" s="50" t="n">
+      <c r="C15" s="51" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="50" t="n">
+      <c r="D15" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="50" t="n">
+      <c r="E15" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="50" t="n">
+      <c r="F15" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="50" t="n">
+      <c r="G15" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="50" t="n">
+      <c r="H15" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="I15" s="54">
+      <c r="I15" s="55">
         <f>3/B15</f>
         <v/>
       </c>
-      <c r="J15" s="50" t="n">
+      <c r="J15" s="51" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
-      <c r="A16" s="50" t="inlineStr">
+      <c r="A16" s="51" t="inlineStr">
         <is>
           <t>15. Non-functional</t>
         </is>
       </c>
-      <c r="B16" s="50" t="n">
+      <c r="B16" s="51" t="n">
         <v>4</v>
       </c>
-      <c r="C16" s="50" t="n">
+      <c r="C16" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="50" t="n">
+      <c r="D16" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="50" t="n">
+      <c r="E16" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="50" t="n">
+      <c r="F16" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="50" t="n">
+      <c r="G16" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="H16" s="50" t="n">
+      <c r="H16" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="54">
+      <c r="I16" s="55">
         <f>3/B16</f>
         <v/>
       </c>
-      <c r="J16" s="50" t="n">
+      <c r="J16" s="51" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="25">
-      <c r="A17" s="50" t="inlineStr">
+      <c r="A17" s="51" t="inlineStr">
         <is>
           <t>16. Event tracking</t>
         </is>
       </c>
-      <c r="B17" s="50" t="n">
+      <c r="B17" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="C17" s="50" t="n">
+      <c r="C17" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="50" t="n">
+      <c r="D17" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="50" t="n">
+      <c r="E17" s="51" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="50" t="n">
+      <c r="F17" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="50" t="n">
+      <c r="G17" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="50" t="n">
+      <c r="H17" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="54">
+      <c r="I17" s="55">
         <f>1/B17</f>
         <v/>
       </c>
-      <c r="J17" s="50" t="n">
+      <c r="J17" s="51" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="25">
-      <c r="A18" s="50" t="inlineStr">
+      <c r="A18" s="51" t="inlineStr">
         <is>
           <t>17. Regression / E2E</t>
         </is>
       </c>
-      <c r="B18" s="50" t="n">
+      <c r="B18" s="51" t="n">
         <v>7</v>
       </c>
-      <c r="C18" s="50" t="n">
+      <c r="C18" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="50" t="n">
+      <c r="D18" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="50" t="n">
+      <c r="E18" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="50" t="n">
+      <c r="F18" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="50" t="n">
+      <c r="G18" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="50" t="n">
+      <c r="H18" s="51" t="n">
         <v>7</v>
       </c>
-      <c r="I18" s="54">
+      <c r="I18" s="55">
         <f>0/B18</f>
         <v/>
       </c>
-      <c r="J18" s="50" t="n">
+      <c r="J18" s="51" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="25">
-      <c r="A19" s="52" t="inlineStr">
+      <c r="A19" s="53" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -11779,7 +11788,7 @@
         <f>SUM(H2:H18)</f>
         <v/>
       </c>
-      <c r="I19" s="55">
+      <c r="I19" s="56">
         <f>76/B19</f>
         <v/>
       </c>
@@ -11855,7 +11864,7 @@
       <c r="A2" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="56" t="inlineStr">
+      <c r="B2" s="57" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -11885,7 +11894,7 @@
       <c r="A3" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="56" t="inlineStr">
+      <c r="B3" s="57" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -11915,7 +11924,7 @@
       <c r="A4" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="56" t="inlineStr">
+      <c r="B4" s="57" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -11945,7 +11954,7 @@
       <c r="A5" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="56" t="inlineStr">
+      <c r="B5" s="57" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -11975,7 +11984,7 @@
       <c r="A6" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="57" t="inlineStr">
+      <c r="B6" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12005,7 +12014,7 @@
       <c r="A7" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="57" t="inlineStr">
+      <c r="B7" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12035,7 +12044,7 @@
       <c r="A8" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="57" t="inlineStr">
+      <c r="B8" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12065,7 +12074,7 @@
       <c r="A9" s="33" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="57" t="inlineStr">
+      <c r="B9" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12095,7 +12104,7 @@
       <c r="A10" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="57" t="inlineStr">
+      <c r="B10" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12125,7 +12134,7 @@
       <c r="A11" s="33" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="57" t="inlineStr">
+      <c r="B11" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12155,7 +12164,7 @@
       <c r="A12" s="33" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="57" t="inlineStr">
+      <c r="B12" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12185,7 +12194,7 @@
       <c r="A13" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="57" t="inlineStr">
+      <c r="B13" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12215,7 +12224,7 @@
       <c r="A14" s="33" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="57" t="inlineStr">
+      <c r="B14" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12245,7 +12254,7 @@
       <c r="A15" s="33" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="57" t="inlineStr">
+      <c r="B15" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12275,7 +12284,7 @@
       <c r="A16" s="33" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="57" t="inlineStr">
+      <c r="B16" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12305,7 +12314,7 @@
       <c r="A17" s="33" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="57" t="inlineStr">
+      <c r="B17" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12335,7 +12344,7 @@
       <c r="A18" s="33" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="57" t="inlineStr">
+      <c r="B18" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12365,7 +12374,7 @@
       <c r="A19" s="33" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="58" t="inlineStr">
+      <c r="B19" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12395,7 +12404,7 @@
       <c r="A20" s="33" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="58" t="inlineStr">
+      <c r="B20" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12425,7 +12434,7 @@
       <c r="A21" s="33" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="58" t="inlineStr">
+      <c r="B21" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12455,7 +12464,7 @@
       <c r="A22" s="33" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="59" t="inlineStr">
+      <c r="B22" s="60" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
@@ -12485,7 +12494,7 @@
       <c r="A23" s="33" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="58" t="inlineStr">
+      <c r="B23" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12515,7 +12524,7 @@
       <c r="A24" s="33" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="58" t="inlineStr">
+      <c r="B24" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12545,7 +12554,7 @@
       <c r="A25" s="33" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="58" t="inlineStr">
+      <c r="B25" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12575,7 +12584,7 @@
       <c r="A26" s="33" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="58" t="inlineStr">
+      <c r="B26" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12605,7 +12614,7 @@
       <c r="A27" s="33" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="58" t="inlineStr">
+      <c r="B27" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12635,7 +12644,7 @@
       <c r="A28" s="33" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="58" t="inlineStr">
+      <c r="B28" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12665,7 +12674,7 @@
       <c r="A29" s="33" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="58" t="inlineStr">
+      <c r="B29" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12695,7 +12704,7 @@
       <c r="A30" s="33" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="59" t="inlineStr">
+      <c r="B30" s="60" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
@@ -12725,7 +12734,7 @@
       <c r="A31" s="33" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="58" t="inlineStr">
+      <c r="B31" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12755,7 +12764,7 @@
       <c r="A32" s="33" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="57" t="inlineStr">
+      <c r="B32" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12785,7 +12794,7 @@
       <c r="A33" s="33" t="n">
         <v>33</v>
       </c>
-      <c r="B33" s="57" t="inlineStr">
+      <c r="B33" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12815,7 +12824,7 @@
       <c r="A34" s="33" t="n">
         <v>34</v>
       </c>
-      <c r="B34" s="57" t="inlineStr">
+      <c r="B34" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12845,7 +12854,7 @@
       <c r="A35" s="33" t="n">
         <v>35</v>
       </c>
-      <c r="B35" s="57" t="inlineStr">
+      <c r="B35" s="58" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12875,7 +12884,7 @@
       <c r="A36" s="33" t="n">
         <v>36</v>
       </c>
-      <c r="B36" s="58" t="inlineStr">
+      <c r="B36" s="59" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12912,4 +12921,464 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" style="25" min="1" max="1"/>
+    <col width="36" customWidth="1" style="25" min="2" max="2"/>
+    <col width="70" customWidth="1" style="25" min="3" max="3"/>
+    <col width="90" customWidth="1" style="25" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B1" s="29" t="inlineStr">
+        <is>
+          <t>Nhóm</t>
+        </is>
+      </c>
+      <c r="C1" s="29" t="inlineStr">
+        <is>
+          <t>Sub-scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="29" t="inlineStr">
+        <is>
+          <t>Lý do bỏ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3. 413 My Balance</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>get_info trả lỗi 5xx khi vào 413</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4. Trừ lượt khi Gen (AC1)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Request gen gửi App User ID, không gửi số dư</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4. Trừ lượt khi Gen (AC1)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>S11 — Leave Anyway rồi vendor trả fail: KHÔNG hoàn lượt [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4. Trừ lượt khi Gen (AC1)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>S5 — Gen fail do service lỗi: hoàn về ví topup đã khoá [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4. Trừ lượt khi Gen (AC1)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>S5 — Gen fail do service lỗi: hoàn về ví quota đã khoá [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>4. Trừ lượt khi Gen (AC1)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Gen fail do timeout vendor: hoàn lượt [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>4. Trừ lượt khi Gen (AC1)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Thiếu App User ID trong request → ERR16 [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>4. Trừ lượt khi Gen (AC1)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Concurrency — còn 1 lượt, bắn 2+ request cùng lúc qua API [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>6. Màn topup &amp; mua Topup (AC2)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tin báo RevenueCat về chậm — app gọi confirm, BE hỏi thẳng RevenueCat [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>6. Màn topup &amp; mua Topup (AC2)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Webhook đến sau / đến 2 lần — không cộng trùng [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>7. Luồng Free user (AC3)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Gen fail sau khi dùng topup — hoàn lượt, retry chạy lại đủ chuỗi paywall [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>9. Reset quota hằng ngày</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Gen submit trước mốc ở ví topup, fail sau mốc — luôn hoàn [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12. Cấu hình số lượt/ngày trên CMS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Firebase RC không còn key daily_quota_amount — app lấy Q từ BE</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10: case cần PO đổi số lượt/ngày (Q) trên CMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>12. Cấu hình số lượt/ngày trên CMS</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PO đặt số lượt hợp lệ trên CMS — áp dụng sau reset</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10: case cần PO đổi số lượt/ngày (Q) trên CMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>12. Cấu hình số lượt/ngày trên CMS</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Copy số lượt/ngày lấy theo giá trị CMS</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10: case cần PO đổi số lượt/ngày (Q) trên CMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>15. Non-functional</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Offering chỉ tải khi mở màn bán</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>159</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15. Non-functional</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Không prefetch offering topup / last-chance lúc launch &amp; onboarding</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>15. Non-functional</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Request gen thiếu x-api-token bị từ chối [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>173</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>17. Regression / E2E</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ERR12 chỉ còn nghĩa hết lượt [Cần BE hỗ trợ]</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Chấm từ bằng chứng/code: Bỏ theo yêu cầu user 25/10 13:34: case cần giả lập phía server (vendor lỗi/timeout, webhook, gọi API trực tiếp, 5xx, proxy) — không thuộc phạm vi autotest app.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>